<commit_message>
print2Excel recursive functions not working
</commit_message>
<xml_diff>
--- a/shipClassTests/sensed_system_output.xlsx
+++ b/shipClassTests/sensed_system_output.xlsx
@@ -14,9 +14,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Time Step</t>
+  </si>
+  <si>
+    <t>Sys Truth State</t>
+  </si>
+  <si>
+    <t>Component_1 Truth State</t>
+  </si>
+  <si>
+    <t>Component_2 Truth State</t>
+  </si>
+  <si>
+    <t>Component_3 Truth State</t>
+  </si>
+  <si>
+    <t>Component_4 Truth State</t>
+  </si>
+  <si>
+    <t>Component_5 Truth State</t>
+  </si>
+  <si>
+    <t>Sys Sensed State</t>
+  </si>
+  <si>
+    <t>Component_1 Sensed State</t>
+  </si>
+  <si>
+    <t>Component_2 Sensed State</t>
+  </si>
+  <si>
+    <t>Component_3 Sensed State</t>
+  </si>
+  <si>
+    <t>Component_4 Sensed State</t>
+  </si>
+  <si>
+    <t>Component_5 Sensed State</t>
+  </si>
+  <si>
+    <t>Does Sensed State Match Truth State?</t>
   </si>
 </sst>
 </file>
@@ -48,27 +87,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -84,19 +108,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC0C0C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00FFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -386,20 +429,1277 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="15" width="12.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="3">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2" s="4">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3">
+        <f>IF(B2 = H2, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="4">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3">
+        <f>IF(B3 = H3, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3">
+        <f>IF(B4 = H4, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4">
+        <v>0</v>
+      </c>
+      <c r="N5" s="3">
+        <f>IF(B5 = H5, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4">
+        <v>0</v>
+      </c>
+      <c r="N6" s="3">
+        <f>IF(B6 = H6, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0</v>
+      </c>
+      <c r="N7" s="3">
+        <f>IF(B7 = H7, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4">
+        <v>0</v>
+      </c>
+      <c r="N8" s="3">
+        <f>IF(B8 = H8, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>2</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4">
+        <v>0</v>
+      </c>
+      <c r="N9" s="3">
+        <f>IF(B9 = H9, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3">
+        <f>IF(B10 = H10, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4">
+        <v>0</v>
+      </c>
+      <c r="N11" s="3">
+        <f>IF(B11 = H11, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>2</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4">
+        <v>0</v>
+      </c>
+      <c r="N12" s="3">
+        <f>IF(B12 = H12, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4">
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <f>IF(B13 = H13, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14" s="4">
+        <v>0</v>
+      </c>
+      <c r="N14" s="3">
+        <f>IF(B14 = H14, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4">
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <f>IF(B15 = H15, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4">
+        <v>0</v>
+      </c>
+      <c r="N16" s="3">
+        <f>IF(B16 = H16, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17" s="4">
+        <v>0</v>
+      </c>
+      <c r="N17" s="3">
+        <f>IF(B17 = H17, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18" s="4">
+        <v>0</v>
+      </c>
+      <c r="N18" s="3">
+        <f>IF(B18 = H18, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4">
+        <v>0</v>
+      </c>
+      <c r="N19" s="3">
+        <f>IF(B19 = H19, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4">
+        <v>0</v>
+      </c>
+      <c r="N20" s="3">
+        <f>IF(B20 = H20, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4">
+        <v>0</v>
+      </c>
+      <c r="N21" s="3">
+        <f>IF(B21 = H21, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22" s="4">
+        <v>0</v>
+      </c>
+      <c r="N22" s="3">
+        <f>IF(B22 = H22, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3">
+        <f>IF(B23 = H23, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4">
+        <v>0</v>
+      </c>
+      <c r="N24" s="3">
+        <f>IF(B24 = H24, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4">
+        <v>0</v>
+      </c>
+      <c r="N25" s="3">
+        <f>IF(B25 = H25, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>2</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4">
+        <v>0</v>
+      </c>
+      <c r="N26" s="3">
+        <f>IF(B26 = H26, 1, 0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="4">
+        <v>0</v>
+      </c>
+      <c r="N27" s="3">
+        <f>IF(B27 = H27, 1, 0)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C28">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="2">
+      <formula>LEN(TRIM(C2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D28">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(D2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F28">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="4">
+      <formula>LEN(TRIM(F2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G28">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="5">
+      <formula>LEN(TRIM(G2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I28">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="6">
+      <formula>LEN(TRIM(I2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J28">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="7">
+      <formula>LEN(TRIM(J2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L28">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="8">
+      <formula>LEN(TRIM(L2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M28">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="9">
+      <formula>LEN(TRIM(M2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N27">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFD0000"/>
+        <color rgb="FF00FD00"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>